<commit_message>
updated sample excel file
</commit_message>
<xml_diff>
--- a/assets/Communicate_Pro__Essential_Conversations__20260314_1410Z.xlsx
+++ b/assets/Communicate_Pro__Essential_Conversations__20260314_1410Z.xlsx
@@ -1,27 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5EC022-4EAE-40FB-BC05-6B1A96479A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="18072" windowHeight="12156" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Training Program" sheetId="1" r:id="rId1"/>
-    <sheet name="Options" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Training Program" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Options" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="155">
   <si>
     <t>Product</t>
   </si>
@@ -56,7 +47,7 @@
     <t>Media</t>
   </si>
   <si>
-    <t>Type of Content</t>
+    <t>Content Type</t>
   </si>
   <si>
     <t>Duration</t>
@@ -71,6 +62,9 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Engage360</t>
+  </si>
+  <si>
     <t>Essential Conversations</t>
   </si>
   <si>
@@ -92,10 +86,13 @@
     <t>Self-Paced</t>
   </si>
   <si>
-    <t>Web Article</t>
-  </si>
-  <si>
-    <t>Facts/ Concepts</t>
+    <t>Online Article / Web Page</t>
+  </si>
+  <si>
+    <t>Facts / Concepts</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Keep</t>
@@ -125,10 +122,10 @@
     <t>Scenario-Based Exercise</t>
   </si>
   <si>
-    <t>Activity Sheets</t>
-  </si>
-  <si>
-    <t>Problem-Solving - Customer Service</t>
+    <t>Activity Sheet / Workbook</t>
+  </si>
+  <si>
+    <t>Problem-Solving - Communication Skills</t>
   </si>
   <si>
     <t>Active Listening Essentials</t>
@@ -137,7 +134,7 @@
     <t>Recognize the behaviors of active listening (paraphrase, reflect emotion, summarize, confirm).</t>
   </si>
   <si>
-    <t>Watching</t>
+    <t>Video / Recording Review</t>
   </si>
   <si>
     <t>Produced Instructional Video</t>
@@ -146,16 +143,16 @@
     <t>Apply listening techniques in structured pair drills with timed prompts.</t>
   </si>
   <si>
-    <t>Workshop</t>
-  </si>
-  <si>
-    <t>Procedural - Customer Service</t>
+    <t>Facilitated Group Activity</t>
+  </si>
+  <si>
+    <t>Procedural - Communication Skills</t>
   </si>
   <si>
     <t>Demonstrate active listening in a short role play and receive peer feedback.</t>
   </si>
   <si>
-    <t>Role Play/ Mock Call Exercise</t>
+    <t>Role Play / Mock Conversation</t>
   </si>
   <si>
     <t>Questioning and Clarifying Needs</t>
@@ -164,10 +161,10 @@
     <t>Recall common question types (open, closed, probing, clarifying) and when to use each.</t>
   </si>
   <si>
-    <t>Module Interaction</t>
-  </si>
-  <si>
-    <t>eLearning</t>
+    <t>eLearning - Interactive</t>
+  </si>
+  <si>
+    <t>eLearning Module</t>
   </si>
   <si>
     <t>Draft a question funnel for a common workplace situation (from broad to specific).</t>
@@ -185,7 +182,7 @@
     <t>Summarize key concepts from communication barriers, listening, and questioning.</t>
   </si>
   <si>
-    <t>Recap/ Debrief</t>
+    <t>Recap &amp; Debrief</t>
   </si>
   <si>
     <t>Verbal &amp; Non-Verbal Communication</t>
@@ -272,7 +269,7 @@
     <t>Recall channel norms (when to use chat vs email vs meeting) and expected response times.</t>
   </si>
   <si>
-    <t>Workflow - Operations/ Admin/ Support</t>
+    <t>Workflow - Operations / Admin / Support</t>
   </si>
   <si>
     <t>Build a team communication agreement (channels, turnaround times, escalation triggers).</t>
@@ -290,7 +287,7 @@
     <t>Revise your draft using peer comments and finalize a professional version.</t>
   </si>
   <si>
-    <t>Online Notebook</t>
+    <t>Digital Workspace / Notebook</t>
   </si>
   <si>
     <t>Day 3 Recap</t>
@@ -341,7 +338,7 @@
     <t>Perform a structured difficult-conversation simulation observed by facilitator.</t>
   </si>
   <si>
-    <t>Graded Mock Calls</t>
+    <t>Graded Practice Conversation</t>
   </si>
   <si>
     <t>Evaluate peer simulations using the rubric and identify decision points that mattered most.</t>
@@ -350,140 +347,149 @@
     <t>Summarize capstone takeaways and create a 2-week action plan with measurable behaviors.</t>
   </si>
   <si>
-    <t>Cognitive Tasks</t>
-  </si>
-  <si>
-    <t>Delivery Methods</t>
+    <t>eLearning - Read, Watch, Listen</t>
   </si>
   <si>
     <t>Remove</t>
   </si>
   <si>
+    <t>Podcast / Audio Review</t>
+  </si>
+  <si>
     <t>On-the-Job Training</t>
   </si>
   <si>
+    <t>Spreadsheet</t>
+  </si>
+  <si>
+    <t>Procedural - Software / Tools</t>
+  </si>
+  <si>
+    <t>Rebrand</t>
+  </si>
+  <si>
+    <t>Microlearning</t>
+  </si>
+  <si>
     <t>Text Document</t>
   </si>
   <si>
-    <t>Procedural - Software/ Tools</t>
-  </si>
-  <si>
-    <t>Rebrand</t>
-  </si>
-  <si>
-    <t>Microlearning</t>
-  </si>
-  <si>
-    <t>Spreadsheet</t>
-  </si>
-  <si>
     <t>Minor Change</t>
   </si>
   <si>
-    <t>Problem-Solving - Software/ Tools</t>
+    <t>Infographic / Visual Aid</t>
+  </si>
+  <si>
+    <t>Problem-Solving - Software / Tools</t>
   </si>
   <si>
     <t>Major Update</t>
   </si>
   <si>
-    <t>Listening</t>
+    <t>Concept Mapping / Mind Mapping</t>
   </si>
   <si>
     <t>Merge w/ Below</t>
   </si>
   <si>
-    <t>Navigation Practice</t>
-  </si>
-  <si>
-    <t>Graphics</t>
+    <t>Audio Recording / Podcast</t>
   </si>
   <si>
     <t>Add to Above</t>
   </si>
   <si>
+    <t>Split</t>
+  </si>
+  <si>
+    <t>Pre-Training / Advance Organizer</t>
+  </si>
+  <si>
+    <t>Recorded Lecture</t>
+  </si>
+  <si>
+    <t>New Addition</t>
+  </si>
+  <si>
+    <t>Q&amp;A with Instructor / Expert</t>
+  </si>
+  <si>
+    <t>Live System / Application</t>
+  </si>
+  <si>
     <t>Documentation Practice</t>
   </si>
   <si>
-    <t>Audio Recording/ Podcast</t>
-  </si>
-  <si>
-    <t>Split</t>
-  </si>
-  <si>
-    <t>Reference/ Job Aids Practice</t>
-  </si>
-  <si>
-    <t>Recorded Lecture</t>
-  </si>
-  <si>
-    <t>New Addition</t>
-  </si>
-  <si>
-    <t>Interactive Q&amp;A</t>
-  </si>
-  <si>
-    <t>Quiz/ Survey</t>
-  </si>
-  <si>
-    <t>Tool/ Software</t>
+    <t>Quiz / Survey</t>
+  </si>
+  <si>
+    <t>eLearning - Simulate &amp; Practice</t>
   </si>
   <si>
     <t>Collaborative Platform</t>
   </si>
   <si>
+    <t>Job Aid &amp; Reference Lookup Practice</t>
+  </si>
+  <si>
+    <t>Shadowing &amp; Job Observation</t>
+  </si>
+  <si>
+    <t>Guest Speaker / SME Session</t>
+  </si>
+  <si>
+    <t>Software / Tool Practice</t>
+  </si>
+  <si>
+    <t>VR / AR</t>
+  </si>
+  <si>
+    <t>Worked Example Review</t>
+  </si>
+  <si>
     <t>Asynchronous Group Discussion</t>
   </si>
   <si>
+    <t>Live Customer Practice</t>
+  </si>
+  <si>
+    <t>Mentorship / Coaching</t>
+  </si>
+  <si>
     <t>Peer Teaching</t>
   </si>
   <si>
-    <t>Subject Matter Expert</t>
-  </si>
-  <si>
-    <t>VR/AR</t>
-  </si>
-  <si>
     <t>Knowledge Check</t>
   </si>
   <si>
+    <t>Procedural Skills Assessment</t>
+  </si>
+  <si>
+    <t>Self Assessment</t>
+  </si>
+  <si>
     <t>Written Graded Assessment</t>
   </si>
   <si>
-    <t>Navigation Assessment</t>
-  </si>
-  <si>
-    <t>Self Assessment</t>
-  </si>
-  <si>
-    <t>Shadowing/ Observation</t>
-  </si>
-  <si>
-    <t>Live Customer Practice</t>
-  </si>
-  <si>
-    <t>Mentorship/ Coaching</t>
-  </si>
-  <si>
-    <t>Game</t>
+    <t>Ice Breaker</t>
+  </si>
+  <si>
+    <t>Learning Game</t>
   </si>
   <si>
     <t>Meet &amp; Greet</t>
-  </si>
-  <si>
-    <t>Engage360</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -513,7 +519,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -600,6 +606,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -634,6 +641,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -668,20 +676,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -803,17 +807,56 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -863,12 +906,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -877,42 +920,48 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M2">
         <v>15</v>
       </c>
+      <c r="N2" t="s">
+        <v>26</v>
+      </c>
       <c r="O2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -921,42 +970,48 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M3">
         <v>25</v>
       </c>
+      <c r="N3" t="s">
+        <v>26</v>
+      </c>
       <c r="O3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -965,42 +1020,48 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" t="s">
         <v>31</v>
       </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" t="s">
-        <v>29</v>
-      </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M4">
         <v>25</v>
       </c>
+      <c r="N4" t="s">
+        <v>26</v>
+      </c>
       <c r="O4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1009,42 +1070,48 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M5">
         <v>15</v>
       </c>
+      <c r="N5" t="s">
+        <v>26</v>
+      </c>
       <c r="O5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1053,42 +1120,48 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
-      </c>
-      <c r="K6" t="s">
-        <v>34</v>
-      </c>
       <c r="L6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M6">
         <v>30</v>
       </c>
+      <c r="N6" t="s">
+        <v>26</v>
+      </c>
       <c r="O6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1097,42 +1170,48 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" t="s">
         <v>36</v>
       </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="L7" t="s">
         <v>44</v>
-      </c>
-      <c r="J7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" t="s">
-        <v>34</v>
-      </c>
-      <c r="L7" t="s">
-        <v>42</v>
       </c>
       <c r="M7">
         <v>30</v>
       </c>
+      <c r="N7" t="s">
+        <v>26</v>
+      </c>
       <c r="O7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1141,42 +1220,48 @@
         <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M8">
         <v>15</v>
       </c>
+      <c r="N8" t="s">
+        <v>26</v>
+      </c>
       <c r="O8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1185,42 +1270,48 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M9">
         <v>25</v>
       </c>
+      <c r="N9" t="s">
+        <v>26</v>
+      </c>
       <c r="O9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1229,42 +1320,48 @@
         <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="J10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M10">
         <v>30</v>
       </c>
+      <c r="N10" t="s">
+        <v>26</v>
+      </c>
       <c r="O10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1273,42 +1370,48 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M11">
         <v>30</v>
       </c>
+      <c r="N11" t="s">
+        <v>26</v>
+      </c>
       <c r="O11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1317,42 +1420,48 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M12">
         <v>15</v>
       </c>
+      <c r="N12" t="s">
+        <v>26</v>
+      </c>
       <c r="O12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -1361,42 +1470,48 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M13">
         <v>25</v>
       </c>
+      <c r="N13" t="s">
+        <v>26</v>
+      </c>
       <c r="O13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -1405,42 +1520,48 @@
         <v>3</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M14">
         <v>25</v>
       </c>
+      <c r="N14" t="s">
+        <v>26</v>
+      </c>
       <c r="O14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -1449,42 +1570,48 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M15">
         <v>15</v>
       </c>
+      <c r="N15" t="s">
+        <v>26</v>
+      </c>
       <c r="O15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -1493,42 +1620,48 @@
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M16">
         <v>25</v>
       </c>
+      <c r="N16" t="s">
+        <v>26</v>
+      </c>
       <c r="O16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -1537,42 +1670,48 @@
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G17" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I17" t="s">
+        <v>46</v>
+      </c>
+      <c r="J17" t="s">
+        <v>31</v>
+      </c>
+      <c r="K17" t="s">
+        <v>36</v>
+      </c>
+      <c r="L17" t="s">
         <v>44</v>
-      </c>
-      <c r="J17" t="s">
-        <v>29</v>
-      </c>
-      <c r="K17" t="s">
-        <v>34</v>
-      </c>
-      <c r="L17" t="s">
-        <v>42</v>
       </c>
       <c r="M17">
         <v>30</v>
       </c>
+      <c r="N17" t="s">
+        <v>26</v>
+      </c>
       <c r="O17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -1581,42 +1720,48 @@
         <v>7</v>
       </c>
       <c r="E18" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G18" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M18">
         <v>15</v>
       </c>
+      <c r="N18" t="s">
+        <v>26</v>
+      </c>
       <c r="O18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -1625,42 +1770,48 @@
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M19">
         <v>30</v>
       </c>
+      <c r="N19" t="s">
+        <v>26</v>
+      </c>
       <c r="O19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -1669,42 +1820,48 @@
         <v>9</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F20" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M20">
         <v>30</v>
       </c>
+      <c r="N20" t="s">
+        <v>26</v>
+      </c>
       <c r="O20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -1713,42 +1870,48 @@
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K21" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M21">
         <v>30</v>
       </c>
+      <c r="N21" t="s">
+        <v>26</v>
+      </c>
       <c r="O21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C22">
         <v>3</v>
@@ -1757,42 +1920,48 @@
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G22" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J22" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M22">
         <v>15</v>
       </c>
+      <c r="N22" t="s">
+        <v>26</v>
+      </c>
       <c r="O22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23">
         <v>3</v>
@@ -1801,42 +1970,48 @@
         <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H23" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I23" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M23">
         <v>25</v>
       </c>
+      <c r="N23" t="s">
+        <v>26</v>
+      </c>
       <c r="O23" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24">
         <v>3</v>
@@ -1845,42 +2020,48 @@
         <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F24" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G24" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H24" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I24" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K24" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L24" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M24">
         <v>15</v>
       </c>
+      <c r="N24" t="s">
+        <v>26</v>
+      </c>
       <c r="O24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25">
         <v>3</v>
@@ -1889,42 +2070,48 @@
         <v>4</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F25" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G25" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H25" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I25" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J25" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M25">
         <v>25</v>
       </c>
+      <c r="N25" t="s">
+        <v>26</v>
+      </c>
       <c r="O25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C26">
         <v>3</v>
@@ -1933,42 +2120,48 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F26" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G26" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I26" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="J26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K26" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L26" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M26">
         <v>20</v>
       </c>
+      <c r="N26" t="s">
+        <v>26</v>
+      </c>
       <c r="O26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C27">
         <v>3</v>
@@ -1977,42 +2170,48 @@
         <v>6</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I27" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M27">
         <v>15</v>
       </c>
+      <c r="N27" t="s">
+        <v>26</v>
+      </c>
       <c r="O27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C28">
         <v>3</v>
@@ -2021,42 +2220,48 @@
         <v>7</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G28" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I28" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J28" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K28" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L28" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M28">
         <v>25</v>
       </c>
+      <c r="N28" t="s">
+        <v>26</v>
+      </c>
       <c r="O28" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C29">
         <v>3</v>
@@ -2065,42 +2270,48 @@
         <v>8</v>
       </c>
       <c r="E29" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F29" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H29" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I29" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J29" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M29">
         <v>20</v>
       </c>
+      <c r="N29" t="s">
+        <v>26</v>
+      </c>
       <c r="O29" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C30">
         <v>3</v>
@@ -2109,42 +2320,48 @@
         <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F30" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G30" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I30" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J30" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K30" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L30" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M30">
         <v>25</v>
       </c>
+      <c r="N30" t="s">
+        <v>26</v>
+      </c>
       <c r="O30" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B31" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C31">
         <v>3</v>
@@ -2153,42 +2370,48 @@
         <v>10</v>
       </c>
       <c r="E31" t="s">
+        <v>75</v>
+      </c>
+      <c r="F31" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" t="s">
+        <v>93</v>
+      </c>
+      <c r="H31" t="s">
+        <v>29</v>
+      </c>
+      <c r="I31" t="s">
+        <v>72</v>
+      </c>
+      <c r="J31" t="s">
+        <v>31</v>
+      </c>
+      <c r="K31" t="s">
         <v>73</v>
       </c>
-      <c r="F31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G31" t="s">
-        <v>91</v>
-      </c>
-      <c r="H31" t="s">
-        <v>27</v>
-      </c>
-      <c r="I31" t="s">
-        <v>70</v>
-      </c>
-      <c r="J31" t="s">
-        <v>29</v>
-      </c>
-      <c r="K31" t="s">
-        <v>71</v>
-      </c>
       <c r="L31" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M31">
         <v>25</v>
       </c>
+      <c r="N31" t="s">
+        <v>26</v>
+      </c>
       <c r="O31" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32">
         <v>3</v>
@@ -2197,42 +2420,48 @@
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F32" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G32" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H32" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I32" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K32" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M32">
         <v>30</v>
       </c>
+      <c r="N32" t="s">
+        <v>26</v>
+      </c>
       <c r="O32" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C33">
         <v>4</v>
@@ -2241,42 +2470,48 @@
         <v>1</v>
       </c>
       <c r="E33" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H33" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I33" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J33" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K33" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L33" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M33">
         <v>15</v>
       </c>
+      <c r="N33" t="s">
+        <v>26</v>
+      </c>
       <c r="O33" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C34">
         <v>4</v>
@@ -2285,42 +2520,48 @@
         <v>2</v>
       </c>
       <c r="E34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F34" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H34" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I34" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J34" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K34" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L34" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M34">
         <v>25</v>
       </c>
+      <c r="N34" t="s">
+        <v>26</v>
+      </c>
       <c r="O34" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C35">
         <v>4</v>
@@ -2329,42 +2570,48 @@
         <v>3</v>
       </c>
       <c r="E35" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F35" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G35" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H35" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I35" t="s">
+        <v>46</v>
+      </c>
+      <c r="J35" t="s">
+        <v>31</v>
+      </c>
+      <c r="K35" t="s">
+        <v>36</v>
+      </c>
+      <c r="L35" t="s">
         <v>44</v>
-      </c>
-      <c r="J35" t="s">
-        <v>29</v>
-      </c>
-      <c r="K35" t="s">
-        <v>34</v>
-      </c>
-      <c r="L35" t="s">
-        <v>42</v>
       </c>
       <c r="M35">
         <v>30</v>
       </c>
+      <c r="N35" t="s">
+        <v>26</v>
+      </c>
       <c r="O35" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C36">
         <v>4</v>
@@ -2373,42 +2620,48 @@
         <v>4</v>
       </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F36" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H36" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I36" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K36" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L36" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M36">
         <v>15</v>
       </c>
+      <c r="N36" t="s">
+        <v>26</v>
+      </c>
       <c r="O36" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C37">
         <v>4</v>
@@ -2417,42 +2670,48 @@
         <v>5</v>
       </c>
       <c r="E37" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G37" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H37" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I37" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J37" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K37" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L37" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M37">
         <v>25</v>
       </c>
+      <c r="N37" t="s">
+        <v>26</v>
+      </c>
       <c r="O37" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P37" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C38">
         <v>4</v>
@@ -2461,42 +2720,48 @@
         <v>6</v>
       </c>
       <c r="E38" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F38" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G38" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H38" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J38" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L38" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M38">
         <v>20</v>
       </c>
+      <c r="N38" t="s">
+        <v>26</v>
+      </c>
       <c r="O38" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C39">
         <v>4</v>
@@ -2505,42 +2770,48 @@
         <v>7</v>
       </c>
       <c r="E39" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F39" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G39" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H39" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I39" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J39" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K39" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L39" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M39">
         <v>15</v>
       </c>
+      <c r="N39" t="s">
+        <v>26</v>
+      </c>
       <c r="O39" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C40">
         <v>4</v>
@@ -2549,42 +2820,48 @@
         <v>8</v>
       </c>
       <c r="E40" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F40" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G40" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H40" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I40" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J40" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K40" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L40" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M40">
         <v>30</v>
       </c>
+      <c r="N40" t="s">
+        <v>26</v>
+      </c>
       <c r="O40" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B41" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C41">
         <v>4</v>
@@ -2593,42 +2870,48 @@
         <v>9</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F41" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G41" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H41" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I41" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J41" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K41" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L41" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M41">
         <v>30</v>
       </c>
+      <c r="N41" t="s">
+        <v>26</v>
+      </c>
       <c r="O41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="P41" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="B42" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C42">
         <v>4</v>
@@ -2637,55 +2920,79 @@
         <v>10</v>
       </c>
       <c r="E42" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F42" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G42" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H42" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I42" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J42" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K42" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L42" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M42">
         <v>35</v>
       </c>
+      <c r="N42" t="s">
+        <v>26</v>
+      </c>
       <c r="O42" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="P42" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <dataValidations count="5">
+    <dataValidation type="list" showErrorMessage="1" errorStyle="error" errorTitle="Invalid value" error="Please select a value from the list" sqref="H2:H1048576">
+      <formula1>Options!$A$2:$A$35</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorStyle="error" errorTitle="Invalid value" error="Please select a value from the list" sqref="I2:I1048576">
+      <formula1>Options!$B$2:$B$35</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorStyle="error" errorTitle="Invalid value" error="Please select a value from the list" sqref="J2:J1048576">
+      <formula1>Options!$C$2:$C$35</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorStyle="error" errorTitle="Invalid value" error="Please select a value from the list" sqref="K2:K1048576">
+      <formula1>Options!$D$2:$D$35</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorStyle="error" errorTitle="Invalid value" error="Please select a value from the list" sqref="L2:L1048576">
+      <formula1>Options!$E$2:$E$35</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>109</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
         <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>110</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
         <v>10</v>
@@ -2697,270 +3004,688 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
         <v>30</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>24</v>
       </c>
-      <c r="F2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
         <v>41</v>
       </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" t="s">
-        <v>83</v>
-      </c>
-      <c r="F3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" t="s">
-        <v>116</v>
-      </c>
-      <c r="D5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>119</v>
-      </c>
-      <c r="F6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>121</v>
-      </c>
-      <c r="D7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D9" t="s">
-        <v>127</v>
+      <c r="E9" t="s">
+        <v>26</v>
       </c>
       <c r="F9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
       <c r="B10" t="s">
         <v>129</v>
       </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
       <c r="D10" t="s">
         <v>130</v>
       </c>
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
       <c r="F10" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
       <c r="B11" t="s">
         <v>132</v>
       </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
       <c r="D11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
       </c>
       <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>70</v>
+      <c r="C14" t="s">
+        <v>26</v>
       </c>
       <c r="D14" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
       <c r="B15" t="s">
         <v>136</v>
       </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
       <c r="D15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
       <c r="B16" t="s">
-        <v>137</v>
+        <v>138</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
       </c>
       <c r="D16" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>145</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" t="s">
+        <v>146</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" t="s">
+        <v>26</v>
+      </c>
+      <c r="F23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B27" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B29" t="s">
-        <v>148</v>
+      <c r="C29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" t="s">
+        <v>149</v>
+      </c>
+      <c r="C30" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" t="s">
+        <v>151</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" t="s">
+        <v>26</v>
+      </c>
+      <c r="F32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" t="s">
+        <v>152</v>
+      </c>
+      <c r="C33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" t="s">
+        <v>26</v>
+      </c>
+      <c r="F33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>